<commit_message>
add age structure, unsure if working
</commit_message>
<xml_diff>
--- a/tests/test_data/south_africa_age_data.xlsx
+++ b/tests/test_data/south_africa_age_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robynstuart/Documents/git/hpvsim/tests/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{438A0348-6E6A-6640-AE5C-B37308AC4450}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEE81852-A394-074C-B47A-20A4D77B8BEA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1180" yWindow="1500" windowWidth="27240" windowHeight="15560" xr2:uid="{5D7E3FBA-9D2B-2843-BAA4-D4EB28E49B52}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -404,9 +404,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C9993B8-80AA-8549-899C-308C8A5037BC}">
   <dimension ref="A1:F153"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="15.5" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -426,7 +429,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2001</v>
       </c>
@@ -446,7 +449,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2001</v>
       </c>
@@ -467,7 +470,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2001</v>
       </c>
@@ -488,7 +491,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2001</v>
       </c>
@@ -509,7 +512,7 @@
         <v>1180</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2001</v>
       </c>
@@ -530,7 +533,7 @@
         <v>1072</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2001</v>
       </c>
@@ -551,7 +554,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2001</v>
       </c>
@@ -572,7 +575,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2001</v>
       </c>
@@ -593,7 +596,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2002</v>
       </c>
@@ -613,7 +616,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2002</v>
       </c>
@@ -634,7 +637,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2002</v>
       </c>
@@ -655,7 +658,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2002</v>
       </c>
@@ -676,7 +679,7 @@
         <v>1193</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2002</v>
       </c>
@@ -697,7 +700,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2002</v>
       </c>
@@ -718,7 +721,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2002</v>
       </c>
@@ -739,7 +742,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2002</v>
       </c>
@@ -760,7 +763,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>2003</v>
       </c>
@@ -780,7 +783,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>2003</v>
       </c>
@@ -801,7 +804,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>2003</v>
       </c>
@@ -822,7 +825,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>2003</v>
       </c>
@@ -843,7 +846,7 @@
         <v>1178</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>2003</v>
       </c>
@@ -864,7 +867,7 @@
         <v>1027</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>2003</v>
       </c>
@@ -885,7 +888,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>2003</v>
       </c>
@@ -906,7 +909,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>2003</v>
       </c>
@@ -927,7 +930,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>2004</v>
       </c>
@@ -947,7 +950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>2004</v>
       </c>
@@ -968,7 +971,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>2004</v>
       </c>
@@ -989,7 +992,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>2004</v>
       </c>
@@ -1010,7 +1013,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>2004</v>
       </c>
@@ -1031,7 +1034,7 @@
         <v>1077</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>2004</v>
       </c>
@@ -1052,7 +1055,7 @@
         <v>847</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>2004</v>
       </c>
@@ -1073,7 +1076,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>2004</v>
       </c>
@@ -1094,7 +1097,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>2005</v>
       </c>
@@ -1114,7 +1117,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>2005</v>
       </c>
@@ -1135,7 +1138,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>2005</v>
       </c>
@@ -1156,7 +1159,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>2005</v>
       </c>
@@ -1177,7 +1180,7 @@
         <v>1207</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>2005</v>
       </c>
@@ -1198,7 +1201,7 @@
         <v>1212</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>2005</v>
       </c>
@@ -1219,7 +1222,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>2005</v>
       </c>
@@ -1240,7 +1243,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>2005</v>
       </c>
@@ -1261,7 +1264,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>2006</v>
       </c>
@@ -1281,7 +1284,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>2006</v>
       </c>
@@ -1302,7 +1305,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="44" spans="1:6">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>2006</v>
       </c>
@@ -1323,7 +1326,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>2006</v>
       </c>
@@ -1344,7 +1347,7 @@
         <v>1254</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>2006</v>
       </c>
@@ -1365,7 +1368,7 @@
         <v>1202</v>
       </c>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>2006</v>
       </c>
@@ -1386,7 +1389,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>2006</v>
       </c>
@@ -1407,7 +1410,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="49" spans="1:6">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>2006</v>
       </c>
@@ -1428,7 +1431,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="50" spans="1:6">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>2007</v>
       </c>
@@ -1448,7 +1451,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:6">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>2007</v>
       </c>
@@ -1469,7 +1472,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="52" spans="1:6">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>2007</v>
       </c>
@@ -1490,7 +1493,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="53" spans="1:6">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>2007</v>
       </c>
@@ -1511,7 +1514,7 @@
         <v>1233</v>
       </c>
     </row>
-    <row r="54" spans="1:6">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>2007</v>
       </c>
@@ -1532,7 +1535,7 @@
         <v>1198</v>
       </c>
     </row>
-    <row r="55" spans="1:6">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>2007</v>
       </c>
@@ -1553,7 +1556,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="56" spans="1:6">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>2007</v>
       </c>
@@ -1574,7 +1577,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="57" spans="1:6">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>2007</v>
       </c>
@@ -1595,7 +1598,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="58" spans="1:6">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>2008</v>
       </c>
@@ -1615,7 +1618,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="1:6">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>2008</v>
       </c>
@@ -1636,7 +1639,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="60" spans="1:6">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>2008</v>
       </c>
@@ -1657,7 +1660,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="61" spans="1:6">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>2008</v>
       </c>
@@ -1678,7 +1681,7 @@
         <v>1287</v>
       </c>
     </row>
-    <row r="62" spans="1:6">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>2008</v>
       </c>
@@ -1699,7 +1702,7 @@
         <v>1174</v>
       </c>
     </row>
-    <row r="63" spans="1:6">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>2008</v>
       </c>
@@ -1720,7 +1723,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="64" spans="1:6">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>2008</v>
       </c>
@@ -1741,7 +1744,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="65" spans="1:6">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>2008</v>
       </c>
@@ -1762,7 +1765,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="66" spans="1:6">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>2009</v>
       </c>
@@ -1782,7 +1785,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="67" spans="1:6">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>2009</v>
       </c>
@@ -1803,7 +1806,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="68" spans="1:6">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>2009</v>
       </c>
@@ -1824,7 +1827,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="69" spans="1:6">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>2009</v>
       </c>
@@ -1845,7 +1848,7 @@
         <v>1334</v>
       </c>
     </row>
-    <row r="70" spans="1:6">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>2009</v>
       </c>
@@ -1866,7 +1869,7 @@
         <v>1250</v>
       </c>
     </row>
-    <row r="71" spans="1:6">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>2009</v>
       </c>
@@ -1887,7 +1890,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="72" spans="1:6">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>2009</v>
       </c>
@@ -1908,7 +1911,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="73" spans="1:6">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>2009</v>
       </c>
@@ -1929,7 +1932,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="74" spans="1:6">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>2010</v>
       </c>
@@ -1949,7 +1952,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="75" spans="1:6">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>2010</v>
       </c>
@@ -1970,7 +1973,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="76" spans="1:6">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>2010</v>
       </c>
@@ -1991,7 +1994,7 @@
         <v>941</v>
       </c>
     </row>
-    <row r="77" spans="1:6">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>2010</v>
       </c>
@@ -2012,7 +2015,7 @@
         <v>1378</v>
       </c>
     </row>
-    <row r="78" spans="1:6">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>2010</v>
       </c>
@@ -2033,7 +2036,7 @@
         <v>1274</v>
       </c>
     </row>
-    <row r="79" spans="1:6">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>2010</v>
       </c>
@@ -2054,7 +2057,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="80" spans="1:6">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>2010</v>
       </c>
@@ -2075,7 +2078,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="81" spans="1:6">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>2010</v>
       </c>
@@ -2096,7 +2099,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="82" spans="1:6">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>2011</v>
       </c>
@@ -2116,7 +2119,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="83" spans="1:6">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>2011</v>
       </c>
@@ -2137,7 +2140,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="84" spans="1:6">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>2011</v>
       </c>
@@ -2158,7 +2161,7 @@
         <v>857</v>
       </c>
     </row>
-    <row r="85" spans="1:6">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>2011</v>
       </c>
@@ -2179,7 +2182,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="86" spans="1:6">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>2011</v>
       </c>
@@ -2200,7 +2203,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="87" spans="1:6">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>2011</v>
       </c>
@@ -2221,7 +2224,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="88" spans="1:6">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>2011</v>
       </c>
@@ -2242,7 +2245,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="89" spans="1:6">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>2011</v>
       </c>
@@ -2263,7 +2266,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="90" spans="1:6">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>2012</v>
       </c>
@@ -2283,7 +2286,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:6">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>2012</v>
       </c>
@@ -2304,7 +2307,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="92" spans="1:6">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>2012</v>
       </c>
@@ -2325,7 +2328,7 @@
         <v>811</v>
       </c>
     </row>
-    <row r="93" spans="1:6">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>2012</v>
       </c>
@@ -2346,7 +2349,7 @@
         <v>1470</v>
       </c>
     </row>
-    <row r="94" spans="1:6">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>2012</v>
       </c>
@@ -2367,7 +2370,7 @@
         <v>1426</v>
       </c>
     </row>
-    <row r="95" spans="1:6">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>2012</v>
       </c>
@@ -2388,7 +2391,7 @@
         <v>947</v>
       </c>
     </row>
-    <row r="96" spans="1:6">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>2012</v>
       </c>
@@ -2409,7 +2412,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="97" spans="1:6">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>2012</v>
       </c>
@@ -2430,7 +2433,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="98" spans="1:6">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>2013</v>
       </c>
@@ -2450,7 +2453,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="99" spans="1:6">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>2013</v>
       </c>
@@ -2471,7 +2474,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="100" spans="1:6">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>2013</v>
       </c>
@@ -2492,7 +2495,7 @@
         <v>1029</v>
       </c>
     </row>
-    <row r="101" spans="1:6">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>2013</v>
       </c>
@@ -2513,7 +2516,7 @@
         <v>1396</v>
       </c>
     </row>
-    <row r="102" spans="1:6">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>2013</v>
       </c>
@@ -2534,7 +2537,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="103" spans="1:6">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>2013</v>
       </c>
@@ -2555,7 +2558,7 @@
         <v>875</v>
       </c>
     </row>
-    <row r="104" spans="1:6">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>2013</v>
       </c>
@@ -2576,7 +2579,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="105" spans="1:6">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>2013</v>
       </c>
@@ -2597,7 +2600,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="106" spans="1:6">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>2014</v>
       </c>
@@ -2617,7 +2620,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="107" spans="1:6">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>2014</v>
       </c>
@@ -2638,7 +2641,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="108" spans="1:6">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>2014</v>
       </c>
@@ -2659,7 +2662,7 @@
         <v>1033</v>
       </c>
     </row>
-    <row r="109" spans="1:6">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>2014</v>
       </c>
@@ -2680,7 +2683,7 @@
         <v>1448</v>
       </c>
     </row>
-    <row r="110" spans="1:6">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>2014</v>
       </c>
@@ -2701,7 +2704,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="111" spans="1:6">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>2014</v>
       </c>
@@ -2722,7 +2725,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="112" spans="1:6">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>2014</v>
       </c>
@@ -2743,7 +2746,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="113" spans="1:6">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>2014</v>
       </c>
@@ -2764,7 +2767,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="114" spans="1:6">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>2015</v>
       </c>
@@ -2784,7 +2787,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="115" spans="1:6">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>2015</v>
       </c>
@@ -2805,7 +2808,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="116" spans="1:6">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>2015</v>
       </c>
@@ -2826,7 +2829,7 @@
         <v>1172</v>
       </c>
     </row>
-    <row r="117" spans="1:6">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>2015</v>
       </c>
@@ -2847,7 +2850,7 @@
         <v>1823</v>
       </c>
     </row>
-    <row r="118" spans="1:6">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>2015</v>
       </c>
@@ -2868,7 +2871,7 @@
         <v>1594</v>
       </c>
     </row>
-    <row r="119" spans="1:6">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A119">
         <v>2015</v>
       </c>
@@ -2889,7 +2892,7 @@
         <v>1109</v>
       </c>
     </row>
-    <row r="120" spans="1:6">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120">
         <v>2015</v>
       </c>
@@ -2910,7 +2913,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="121" spans="1:6">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121">
         <v>2015</v>
       </c>
@@ -2930,7 +2933,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="122" spans="1:6">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A122">
         <v>2016</v>
       </c>
@@ -2950,7 +2953,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="123" spans="1:6">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A123">
         <v>2016</v>
       </c>
@@ -2971,7 +2974,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="124" spans="1:6">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124">
         <v>2016</v>
       </c>
@@ -2992,7 +2995,7 @@
         <v>1369</v>
       </c>
     </row>
-    <row r="125" spans="1:6">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125">
         <v>2016</v>
       </c>
@@ -3013,7 +3016,7 @@
         <v>1943</v>
       </c>
     </row>
-    <row r="126" spans="1:6">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126">
         <v>2016</v>
       </c>
@@ -3034,7 +3037,7 @@
         <v>1834</v>
       </c>
     </row>
-    <row r="127" spans="1:6">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A127">
         <v>2016</v>
       </c>
@@ -3055,7 +3058,7 @@
         <v>1205</v>
       </c>
     </row>
-    <row r="128" spans="1:6">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128">
         <v>2016</v>
       </c>
@@ -3076,7 +3079,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="129" spans="1:6">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129">
         <v>2016</v>
       </c>
@@ -3096,7 +3099,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="130" spans="1:6">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130">
         <v>2017</v>
       </c>
@@ -3117,7 +3120,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="131" spans="1:6">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131">
         <v>2017</v>
       </c>
@@ -3138,7 +3141,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="132" spans="1:6">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132">
         <v>2017</v>
       </c>
@@ -3159,7 +3162,7 @@
         <v>1162</v>
       </c>
     </row>
-    <row r="133" spans="1:6">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133">
         <v>2017</v>
       </c>
@@ -3180,7 +3183,7 @@
         <v>1887</v>
       </c>
     </row>
-    <row r="134" spans="1:6">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134">
         <v>2017</v>
       </c>
@@ -3201,7 +3204,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="135" spans="1:6">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135">
         <v>2017</v>
       </c>
@@ -3222,7 +3225,7 @@
         <v>1026</v>
       </c>
     </row>
-    <row r="136" spans="1:6">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136">
         <v>2017</v>
       </c>
@@ -3243,7 +3246,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="137" spans="1:6">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137">
         <v>2017</v>
       </c>
@@ -3263,7 +3266,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="138" spans="1:6">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A138">
         <v>2018</v>
       </c>
@@ -3283,7 +3286,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="139" spans="1:6">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139">
         <v>2018</v>
       </c>
@@ -3304,7 +3307,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="140" spans="1:6">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140">
         <v>2018</v>
       </c>
@@ -3325,7 +3328,7 @@
         <v>1207</v>
       </c>
     </row>
-    <row r="141" spans="1:6">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A141">
         <v>2018</v>
       </c>
@@ -3346,7 +3349,7 @@
         <v>1719</v>
       </c>
     </row>
-    <row r="142" spans="1:6">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142">
         <v>2018</v>
       </c>
@@ -3367,7 +3370,7 @@
         <v>1514</v>
       </c>
     </row>
-    <row r="143" spans="1:6">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143">
         <v>2018</v>
       </c>
@@ -3388,7 +3391,7 @@
         <v>986</v>
       </c>
     </row>
-    <row r="144" spans="1:6">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A144">
         <v>2018</v>
       </c>
@@ -3409,7 +3412,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="145" spans="1:6">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A145">
         <v>2018</v>
       </c>
@@ -3430,7 +3433,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="146" spans="1:6">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A146">
         <v>2019</v>
       </c>
@@ -3450,7 +3453,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="147" spans="1:6">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A147">
         <v>2019</v>
       </c>
@@ -3471,7 +3474,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="148" spans="1:6">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A148">
         <v>2019</v>
       </c>
@@ -3492,7 +3495,7 @@
         <v>1245</v>
       </c>
     </row>
-    <row r="149" spans="1:6">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A149">
         <v>2019</v>
       </c>
@@ -3513,7 +3516,7 @@
         <v>2059</v>
       </c>
     </row>
-    <row r="150" spans="1:6">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150">
         <v>2019</v>
       </c>
@@ -3534,7 +3537,7 @@
         <v>1648</v>
       </c>
     </row>
-    <row r="151" spans="1:6">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A151">
         <v>2019</v>
       </c>
@@ -3555,7 +3558,7 @@
         <v>1169</v>
       </c>
     </row>
-    <row r="152" spans="1:6">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A152">
         <v>2019</v>
       </c>
@@ -3576,7 +3579,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="153" spans="1:6">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A153">
         <v>2019</v>
       </c>

</xml_diff>